<commit_message>
calc few-shot results with a bit better parsing. f single JSON object was malformed - skip only this JSON object (one question)
</commit_message>
<xml_diff>
--- a/src/results/llm/results_for_presentation_few-shot.xlsx
+++ b/src/results/llm/results_for_presentation_few-shot.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\llm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7D534B2-7A0E-47FC-89AE-A8210A202E85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8FDD7D9-5A5F-4251-A6B2-A35FD4E3EB31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="2-shot" sheetId="1" r:id="rId1"/>
+    <sheet name="OG" sheetId="1" r:id="rId1"/>
+    <sheet name="Better Parsing" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="26">
   <si>
     <t>human1</t>
   </si>
@@ -96,6 +97,24 @@
   </si>
   <si>
     <t>Total prompts</t>
+  </si>
+  <si>
+    <t>gemma-26b-q4 OG results (two-shot) without texts 1, 5, 7, 43</t>
+  </si>
+  <si>
+    <t>gemma-26b-q4 OG results (three-shot) without texts  1, 5, 7, 43</t>
+  </si>
+  <si>
+    <t>gemma-26b-q4 OG results (four-shot) without texts  1, 5, 7, 43</t>
+  </si>
+  <si>
+    <t>gemma-26b-q4 OG results (zero-shot) without texts  1, 5, 7, 43</t>
+  </si>
+  <si>
+    <t>Statistics of TOTALLY unparsable JSONs, that were skipped</t>
+  </si>
+  <si>
+    <t>Amount of individual skipped questions</t>
   </si>
 </sst>
 </file>
@@ -127,7 +146,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -200,11 +219,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -214,9 +242,6 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -226,14 +251,43 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -552,23 +606,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="12"/>
-      <c r="I1" s="10" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="11"/>
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="12"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="11"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
@@ -734,23 +788,23 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="12"/>
-      <c r="I8" s="10" t="s">
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="11"/>
+      <c r="I8" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="12"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="11"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
@@ -916,23 +970,23 @@
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="12"/>
-      <c r="I15" s="10" t="s">
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="11"/>
+      <c r="I15" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="12"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="11"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
@@ -1111,22 +1165,22 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9" t="s">
+      <c r="C25" s="12"/>
+      <c r="D25" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9" t="s">
+      <c r="E25" s="12"/>
+      <c r="F25" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="G25" s="9"/>
-      <c r="I25" s="9" t="s">
+      <c r="G25" s="12"/>
+      <c r="I25" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="J25" s="9"/>
+      <c r="J25" s="12"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
@@ -1331,10 +1385,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:G23 G29:G1048576">
-    <cfRule type="cellIs" dxfId="1" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1376,4 +1430,738 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DB0AADD-8776-4402-85B4-2B481E8BF56B}">
+  <dimension ref="A1:N34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" customWidth="1"/>
+    <col min="14" max="14" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="11"/>
+      <c r="I1" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="11"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="2"/>
+      <c r="J2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="6">
+        <v>0.85926928281461401</v>
+      </c>
+      <c r="C3" s="6">
+        <v>0.94494047619047605</v>
+      </c>
+      <c r="D3" s="6">
+        <v>0.90007087172218203</v>
+      </c>
+      <c r="E3" s="6">
+        <v>0.86890770283462404</v>
+      </c>
+      <c r="F3" s="6">
+        <v>0.73877176901924801</v>
+      </c>
+      <c r="G3" s="6">
+        <f>E3-M3</f>
+        <v>2.2674654906410519E-3</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="J3" s="6">
+        <v>0.86164383561643798</v>
+      </c>
+      <c r="K3" s="6">
+        <v>0.93601190476190399</v>
+      </c>
+      <c r="L3" s="6">
+        <v>0.897289586305278</v>
+      </c>
+      <c r="M3" s="6">
+        <v>0.86664023734398299</v>
+      </c>
+      <c r="N3" s="6">
+        <v>0.73400738868364701</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6">
+        <v>0.66949152542372803</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0.90285714285714203</v>
+      </c>
+      <c r="D4" s="6">
+        <v>0.76885644768856398</v>
+      </c>
+      <c r="E4" s="6">
+        <v>0.74832507198181797</v>
+      </c>
+      <c r="F4" s="6">
+        <v>0.50937754824680603</v>
+      </c>
+      <c r="G4" s="6">
+        <f>E4-M4</f>
+        <v>-4.4219885565159878E-3</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="J4" s="6">
+        <v>0.66849315068493098</v>
+      </c>
+      <c r="K4" s="6">
+        <v>0.92952380952380897</v>
+      </c>
+      <c r="L4" s="6">
+        <v>0.777689243027888</v>
+      </c>
+      <c r="M4" s="6">
+        <v>0.75274706053833396</v>
+      </c>
+      <c r="N4" s="6">
+        <v>0.52113821138211303</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="6">
+        <v>0.88219544846050801</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0.89295392953929498</v>
+      </c>
+      <c r="D5" s="6">
+        <v>0.88754208754208697</v>
+      </c>
+      <c r="E5" s="6">
+        <v>0.838739597230163</v>
+      </c>
+      <c r="F5" s="6">
+        <v>0.67750132129934504</v>
+      </c>
+      <c r="G5" s="6">
+        <f>E5-M5</f>
+        <v>8.9722115574879524E-3</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="J5" s="6">
+        <v>0.88356164383561597</v>
+      </c>
+      <c r="K5" s="6">
+        <v>0.87398373983739797</v>
+      </c>
+      <c r="L5" s="6">
+        <v>0.87874659400544897</v>
+      </c>
+      <c r="M5" s="6">
+        <v>0.82976738567267505</v>
+      </c>
+      <c r="N5" s="6">
+        <v>0.65955305013086296</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="11"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="6">
+        <v>0.86516853932584203</v>
+      </c>
+      <c r="C10" s="6">
+        <v>0.91666666666666596</v>
+      </c>
+      <c r="D10" s="6">
+        <v>0.89017341040462405</v>
+      </c>
+      <c r="E10" s="6">
+        <v>0.86026527663088304</v>
+      </c>
+      <c r="F10" s="6">
+        <v>0.72089067573836396</v>
+      </c>
+      <c r="G10" s="6">
+        <f>E10-M3</f>
+        <v>-6.374960713099953E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="6">
+        <v>0.66430594900849804</v>
+      </c>
+      <c r="C11" s="6">
+        <v>0.89333333333333298</v>
+      </c>
+      <c r="D11" s="6">
+        <v>0.76198212835093404</v>
+      </c>
+      <c r="E11" s="6">
+        <v>0.74133424816021398</v>
+      </c>
+      <c r="F11" s="6">
+        <v>0.49546855174913801</v>
+      </c>
+      <c r="G11" s="6">
+        <f t="shared" ref="G11:G12" si="0">E11-M4</f>
+        <v>-1.1412812378119974E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" s="6">
+        <v>0.88423988842398804</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.85907859078590698</v>
+      </c>
+      <c r="D12" s="6">
+        <v>0.87147766323024001</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0.822405498281787</v>
+      </c>
+      <c r="F12" s="6">
+        <v>0.644941439820921</v>
+      </c>
+      <c r="G12" s="6">
+        <f t="shared" si="0"/>
+        <v>-7.3618873908880555E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="11"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B17" s="6">
+        <v>0.85574229691876702</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.90922619047619002</v>
+      </c>
+      <c r="D17" s="6">
+        <v>0.88167388167388105</v>
+      </c>
+      <c r="E17" s="6">
+        <v>0.84911434575864098</v>
+      </c>
+      <c r="F17" s="6">
+        <v>0.69865769215891005</v>
+      </c>
+      <c r="G17" s="6">
+        <f>E17-M3</f>
+        <v>-1.7525891585342013E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="6">
+        <v>0.66911764705882304</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.86666666666666603</v>
+      </c>
+      <c r="D18" s="6">
+        <v>0.755186721991701</v>
+      </c>
+      <c r="E18" s="6">
+        <v>0.74038405867026902</v>
+      </c>
+      <c r="F18" s="6">
+        <v>0.49022282855843502</v>
+      </c>
+      <c r="G18" s="6">
+        <f t="shared" ref="G18:G19" si="1">E18-M4</f>
+        <v>-1.2363001868064938E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B19" s="6">
+        <v>0.878284923928077</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0.86043360433604299</v>
+      </c>
+      <c r="D19" s="6">
+        <v>0.86926762491444198</v>
+      </c>
+      <c r="E19" s="6">
+        <v>0.81802819585160402</v>
+      </c>
+      <c r="F19" s="6">
+        <v>0.63612481450286695</v>
+      </c>
+      <c r="G19" s="6">
+        <f t="shared" si="1"/>
+        <v>-1.1739189821071028E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="13"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="2"/>
+      <c r="B25" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="G25" s="12"/>
+      <c r="I25" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="J25" s="12"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B26" s="2">
+        <v>3</v>
+      </c>
+      <c r="C26" s="6">
+        <f>B26/$J$26</f>
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="D26" s="2">
+        <v>8</v>
+      </c>
+      <c r="E26" s="6">
+        <f>D26/$J$27</f>
+        <v>0.04</v>
+      </c>
+      <c r="F26" s="2">
+        <v>6</v>
+      </c>
+      <c r="G26" s="6">
+        <f>F26/$J$28</f>
+        <v>0.03</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J26" s="2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="2">
+        <v>9</v>
+      </c>
+      <c r="C27" s="6">
+        <f>B27/$J$26</f>
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="D27" s="2">
+        <v>6</v>
+      </c>
+      <c r="E27" s="6">
+        <f>D27/$J$27</f>
+        <v>0.03</v>
+      </c>
+      <c r="F27" s="2">
+        <v>8</v>
+      </c>
+      <c r="G27" s="6">
+        <f>F27/$J$28</f>
+        <v>0.04</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J27" s="2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B28" s="2">
+        <v>2</v>
+      </c>
+      <c r="C28" s="6">
+        <f>B28/$J$26</f>
+        <v>0.01</v>
+      </c>
+      <c r="D28" s="2">
+        <v>8</v>
+      </c>
+      <c r="E28" s="6">
+        <f>D28/$J$27</f>
+        <v>0.04</v>
+      </c>
+      <c r="F28" s="2">
+        <v>4</v>
+      </c>
+      <c r="G28" s="6">
+        <f>F28/$J$28</f>
+        <v>0.02</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J28" s="2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="I30" s="14"/>
+      <c r="J30" s="14"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="2"/>
+      <c r="B31" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B32" s="17">
+        <v>2</v>
+      </c>
+      <c r="C32" s="17">
+        <v>9</v>
+      </c>
+      <c r="D32" s="17">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B33" s="17">
+        <v>0</v>
+      </c>
+      <c r="C33" s="17">
+        <v>4</v>
+      </c>
+      <c r="D33" s="17">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B34" s="17">
+        <v>0</v>
+      </c>
+      <c r="C34" s="17">
+        <v>4</v>
+      </c>
+      <c r="D34" s="17">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="I1:N1"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A15:G15"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B2:G2">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B9:G9">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16:G16">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G1:G23">
+    <cfRule type="cellIs" dxfId="1" priority="5" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="6" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:N2">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
few-shot to csv with json-repair library
</commit_message>
<xml_diff>
--- a/src/results/llm/results_for_presentation_few-shot.xlsx
+++ b/src/results/llm/results_for_presentation_few-shot.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\llm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8FDD7D9-5A5F-4251-A6B2-A35FD4E3EB31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3D38587-311C-4D5D-A227-9ACDD9A49825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OG" sheetId="1" r:id="rId1"/>
     <sheet name="Better Parsing" sheetId="2" r:id="rId2"/>
+    <sheet name="Json-repair" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="26">
   <si>
     <t>human1</t>
   </si>
@@ -232,7 +233,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -242,6 +243,17 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -251,23 +263,101 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="13">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -606,23 +696,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="11"/>
-      <c r="I1" s="9" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="16"/>
+      <c r="I1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="11"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="16"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
@@ -788,23 +878,23 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="11"/>
-      <c r="I8" s="9" t="s">
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="16"/>
+      <c r="I8" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="11"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="16"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
@@ -970,23 +1060,23 @@
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="11"/>
-      <c r="I15" s="9" t="s">
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="16"/>
+      <c r="I15" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="11"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="15"/>
+      <c r="L15" s="15"/>
+      <c r="M15" s="15"/>
+      <c r="N15" s="16"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
@@ -1385,10 +1475,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:G23 G29:G1048576">
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="12" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1451,23 +1541,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="11"/>
-      <c r="I1" s="9" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="16"/>
+      <c r="I1" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="11"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="16"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
@@ -1647,15 +1737,15 @@
       <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="11"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="16"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
@@ -1765,15 +1855,15 @@
       <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="11"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="16"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
@@ -2026,28 +2116,28 @@
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="16" t="s">
+      <c r="A30" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="14"/>
-      <c r="J30" s="14"/>
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+      <c r="J30" s="9"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
-      <c r="B31" s="15" t="s">
+      <c r="B31" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C31" s="15" t="s">
+      <c r="C31" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D31" s="15" t="s">
+      <c r="D31" s="10" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2055,13 +2145,13 @@
       <c r="A32" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B32" s="17">
+      <c r="B32" s="2">
         <v>2</v>
       </c>
-      <c r="C32" s="17">
+      <c r="C32" s="2">
         <v>9</v>
       </c>
-      <c r="D32" s="17">
+      <c r="D32" s="2">
         <v>25</v>
       </c>
     </row>
@@ -2069,13 +2159,13 @@
       <c r="A33" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B33" s="17">
-        <v>0</v>
-      </c>
-      <c r="C33" s="17">
+      <c r="B33" s="2">
+        <v>0</v>
+      </c>
+      <c r="C33" s="2">
         <v>4</v>
       </c>
-      <c r="D33" s="17">
+      <c r="D33" s="2">
         <v>20</v>
       </c>
     </row>
@@ -2083,28 +2173,28 @@
       <c r="A34" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B34" s="17">
-        <v>0</v>
-      </c>
-      <c r="C34" s="17">
+      <c r="B34" s="2">
+        <v>0</v>
+      </c>
+      <c r="C34" s="2">
         <v>4</v>
       </c>
-      <c r="D34" s="17">
+      <c r="D34" s="2">
         <v>22</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="I1:N1"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A15:G15"/>
     <mergeCell ref="A30:D30"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="F25:G25"/>
     <mergeCell ref="I25:J25"/>
-    <mergeCell ref="A24:J24"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="I1:N1"/>
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A15:G15"/>
   </mergeCells>
   <conditionalFormatting sqref="B2:G2">
     <cfRule type="colorScale" priority="7">
@@ -2143,10 +2233,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:G23">
-    <cfRule type="cellIs" dxfId="1" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2164,4 +2254,638 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{762865AC-13CA-4EC7-88AB-2DFC0996DA3B}">
+  <dimension ref="A1:N34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" customWidth="1"/>
+    <col min="10" max="10" width="17.140625" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" customWidth="1"/>
+    <col min="12" max="12" width="13.5703125" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="16"/>
+      <c r="I1" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="16"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="2"/>
+      <c r="J2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6">
+        <f>E3-M3</f>
+        <v>-0.86664023734398299</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="J3" s="6">
+        <v>0.86164383561643798</v>
+      </c>
+      <c r="K3" s="6">
+        <v>0.93601190476190399</v>
+      </c>
+      <c r="L3" s="6">
+        <v>0.897289586305278</v>
+      </c>
+      <c r="M3" s="6">
+        <v>0.86664023734398299</v>
+      </c>
+      <c r="N3" s="6">
+        <v>0.73400738868364701</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6">
+        <f>E4-M4</f>
+        <v>-0.75274706053833396</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="J4" s="6">
+        <v>0.66849315068493098</v>
+      </c>
+      <c r="K4" s="6">
+        <v>0.92952380952380897</v>
+      </c>
+      <c r="L4" s="6">
+        <v>0.777689243027888</v>
+      </c>
+      <c r="M4" s="6">
+        <v>0.75274706053833396</v>
+      </c>
+      <c r="N4" s="6">
+        <v>0.52113821138211303</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6">
+        <f>E5-M5</f>
+        <v>-0.82976738567267505</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="J5" s="6">
+        <v>0.88356164383561597</v>
+      </c>
+      <c r="K5" s="6">
+        <v>0.87398373983739797</v>
+      </c>
+      <c r="L5" s="6">
+        <v>0.87874659400544897</v>
+      </c>
+      <c r="M5" s="6">
+        <v>0.82976738567267505</v>
+      </c>
+      <c r="N5" s="6">
+        <v>0.65955305013086296</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="16"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6">
+        <f>E10-M3</f>
+        <v>-0.86664023734398299</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6">
+        <f t="shared" ref="G11:G12" si="0">E11-M4</f>
+        <v>-0.75274706053833396</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6">
+        <f t="shared" si="0"/>
+        <v>-0.82976738567267505</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="16"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6">
+        <f>E17-M3</f>
+        <v>-0.86664023734398299</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6">
+        <f t="shared" ref="G18:G19" si="1">E18-M4</f>
+        <v>-0.75274706053833396</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6">
+        <f t="shared" si="1"/>
+        <v>-0.82976738567267505</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="13"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="2"/>
+      <c r="B25" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="G25" s="12"/>
+      <c r="I25" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="J25" s="12"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B26" s="2">
+        <v>0</v>
+      </c>
+      <c r="C26" s="6">
+        <f>B26/$J$26</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="2">
+        <v>0</v>
+      </c>
+      <c r="E26" s="6">
+        <f>D26/$J$27</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="2">
+        <v>0</v>
+      </c>
+      <c r="G26" s="6">
+        <f>F26/$J$28</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J26" s="2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="2">
+        <v>0</v>
+      </c>
+      <c r="C27" s="6">
+        <f>B27/$J$26</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="2">
+        <v>0</v>
+      </c>
+      <c r="E27" s="6">
+        <f>D27/$J$27</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="2">
+        <v>0</v>
+      </c>
+      <c r="G27" s="6">
+        <f>F27/$J$28</f>
+        <v>0</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J27" s="2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B28" s="2">
+        <v>1</v>
+      </c>
+      <c r="C28" s="6">
+        <f>B28/$J$26</f>
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="D28" s="2">
+        <v>0</v>
+      </c>
+      <c r="E28" s="6">
+        <f>D28/$J$27</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="2">
+        <v>0</v>
+      </c>
+      <c r="G28" s="6">
+        <f>F28/$J$28</f>
+        <v>0</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J28" s="2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+      <c r="J30" s="9"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="2"/>
+      <c r="B31" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="I1:N1"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="I25:J25"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B2:G2">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B9:G9">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16:G16">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G1:G23">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:N2">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B26:G28">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Calc metric with json-repair results
</commit_message>
<xml_diff>
--- a/src/results/llm/results_for_presentation_few-shot.xlsx
+++ b/src/results/llm/results_for_presentation_few-shot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\llm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3D38587-311C-4D5D-A227-9ACDD9A49825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7527E765-3EA9-4965-B543-312022DE119A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="29">
   <si>
     <t>human1</t>
   </si>
@@ -116,6 +116,15 @@
   </si>
   <si>
     <t>Amount of individual skipped questions</t>
+  </si>
+  <si>
+    <t>Amount of individual skipped invalid JSON objects</t>
+  </si>
+  <si>
+    <t>Amount of times when had to insert default complies=False except those on top</t>
+  </si>
+  <si>
+    <t>Total questions. NB! Approx, because for some texts 1 question in Goal and Tasks might be ommited</t>
   </si>
 </sst>
 </file>
@@ -233,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -248,12 +257,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -263,21 +266,30 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="8">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -300,16 +312,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -325,36 +327,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -696,23 +668,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="16"/>
-      <c r="I1" s="14" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="14"/>
+      <c r="I1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="16"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="14"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
@@ -878,23 +850,23 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="16"/>
-      <c r="I8" s="14" t="s">
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="14"/>
+      <c r="I8" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="J8" s="15"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="15"/>
-      <c r="M8" s="15"/>
-      <c r="N8" s="16"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13"/>
+      <c r="L8" s="13"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="14"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
@@ -1060,23 +1032,23 @@
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="16"/>
-      <c r="I15" s="14" t="s">
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="14"/>
+      <c r="I15" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="J15" s="15"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="15"/>
-      <c r="M15" s="15"/>
-      <c r="N15" s="16"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="13"/>
+      <c r="L15" s="13"/>
+      <c r="M15" s="13"/>
+      <c r="N15" s="14"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
@@ -1242,35 +1214,35 @@
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12" t="s">
+      <c r="C25" s="16"/>
+      <c r="D25" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12" t="s">
+      <c r="E25" s="16"/>
+      <c r="F25" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="G25" s="12"/>
-      <c r="I25" s="12" t="s">
+      <c r="G25" s="16"/>
+      <c r="I25" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="J25" s="12"/>
+      <c r="J25" s="16"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
@@ -1475,10 +1447,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:G23 G29:G1048576">
-    <cfRule type="cellIs" dxfId="12" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1541,23 +1513,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="16"/>
-      <c r="I1" s="14" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="14"/>
+      <c r="I1" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="16"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="14"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
@@ -1737,15 +1709,15 @@
       <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="16"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
@@ -1855,15 +1827,15 @@
       <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="16"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="14"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
@@ -1987,37 +1959,37 @@
       <c r="F23" s="4"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
-      <c r="J24" s="13"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12" t="s">
+      <c r="C25" s="16"/>
+      <c r="D25" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12" t="s">
+      <c r="E25" s="16"/>
+      <c r="F25" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="G25" s="12"/>
-      <c r="I25" s="12" t="s">
+      <c r="G25" s="16"/>
+      <c r="I25" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="J25" s="12"/>
+      <c r="J25" s="16"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
@@ -2185,16 +2157,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="I25:J25"/>
     <mergeCell ref="A24:J24"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="I1:N1"/>
     <mergeCell ref="A8:G8"/>
     <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="I25:J25"/>
   </mergeCells>
   <conditionalFormatting sqref="B2:G2">
     <cfRule type="colorScale" priority="7">
@@ -2233,10 +2205,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:G23">
-    <cfRule type="cellIs" dxfId="10" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2258,7 +2230,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{762865AC-13CA-4EC7-88AB-2DFC0996DA3B}">
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.5703125" customWidth="1"/>
@@ -2275,23 +2247,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="16"/>
-      <c r="I1" s="14" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="14"/>
+      <c r="I1" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="16"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="14"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
@@ -2331,17 +2303,27 @@
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
+      <c r="A3" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="6">
+        <v>0.85885486018641799</v>
+      </c>
+      <c r="C3" s="6">
+        <v>0.95982142857142805</v>
+      </c>
+      <c r="D3" s="6">
+        <v>0.90653548840477804</v>
+      </c>
+      <c r="E3" s="6">
+        <v>0.87567147815804802</v>
+      </c>
+      <c r="F3" s="6">
+        <v>0.75260901063184005</v>
+      </c>
       <c r="G3" s="6">
         <f>E3-M3</f>
-        <v>-0.86664023734398299</v>
+        <v>9.0312408140650335E-3</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>0</v>
@@ -2363,17 +2345,27 @@
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
+      <c r="B4" s="6">
+        <v>0.66352624495289303</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0.93904761904761902</v>
+      </c>
+      <c r="D4" s="6">
+        <v>0.77760252365930604</v>
+      </c>
+      <c r="E4" s="6">
+        <v>0.749473198588546</v>
+      </c>
+      <c r="F4" s="6">
+        <v>0.51684025429460301</v>
+      </c>
       <c r="G4" s="6">
         <f>E4-M4</f>
-        <v>-0.75274706053833396</v>
+        <v>-3.2738619497879595E-3</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>1</v>
@@ -2395,17 +2387,27 @@
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+      <c r="B5" s="6">
+        <v>0.88297872340425498</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0.89972899728997202</v>
+      </c>
+      <c r="D5" s="6">
+        <v>0.89127516778523397</v>
+      </c>
+      <c r="E5" s="6">
+        <v>0.84310593832299696</v>
+      </c>
+      <c r="F5" s="6">
+        <v>0.68626411709544499</v>
+      </c>
       <c r="G5" s="6">
         <f>E5-M5</f>
-        <v>-0.82976738567267505</v>
+        <v>1.3338552650321911E-2</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>2</v>
@@ -2427,32 +2429,36 @@
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="16"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="20"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
+      <c r="A9" s="6"/>
       <c r="B9" s="1" t="s">
         <v>3</v>
       </c>
@@ -2473,74 +2479,108 @@
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
+      <c r="A10" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="6">
+        <v>0.86118598382749301</v>
+      </c>
+      <c r="C10" s="6">
+        <v>0.95089285714285698</v>
+      </c>
+      <c r="D10" s="6">
+        <v>0.90381895332390305</v>
+      </c>
+      <c r="E10" s="6">
+        <v>0.87338753670814095</v>
+      </c>
+      <c r="F10" s="6">
+        <v>0.74778432827079999</v>
+      </c>
       <c r="G10" s="6">
         <f>E10-M3</f>
-        <v>-0.86664023734398299</v>
+        <v>6.7472993641579659E-3</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
+      <c r="B11" s="6">
+        <v>0.66392318244170101</v>
+      </c>
+      <c r="C11" s="6">
+        <v>0.92190476190476101</v>
+      </c>
+      <c r="D11" s="6">
+        <v>0.77192982456140302</v>
+      </c>
+      <c r="E11" s="6">
+        <v>0.74658869395711402</v>
+      </c>
+      <c r="F11" s="6">
+        <v>0.50905723449428497</v>
+      </c>
       <c r="G11" s="6">
         <f t="shared" ref="G11:G12" si="0">E11-M4</f>
-        <v>-0.75274706053833396</v>
+        <v>-6.1583665812199317E-3</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
+      <c r="B12" s="6">
+        <v>0.88651535380507296</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.89972899728997202</v>
+      </c>
+      <c r="D12" s="6">
+        <v>0.89307330195023504</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0.84628444416553295</v>
+      </c>
+      <c r="F12" s="6">
+        <v>0.69260043143799099</v>
+      </c>
       <c r="G12" s="6">
         <f t="shared" si="0"/>
-        <v>-0.82976738567267505</v>
+        <v>1.6517058492857895E-2</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="16"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="20"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
+      <c r="A16" s="6"/>
       <c r="B16" s="1" t="s">
         <v>3</v>
       </c>
@@ -2561,45 +2601,75 @@
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
+      <c r="A17" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B17" s="6">
+        <v>0.85365853658536495</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.9375</v>
+      </c>
+      <c r="D17" s="6">
+        <v>0.89361702127659504</v>
+      </c>
+      <c r="E17" s="6">
+        <v>0.86060161408657299</v>
+      </c>
+      <c r="F17" s="6">
+        <v>0.72218972979295804</v>
+      </c>
       <c r="G17" s="6">
         <f>E17-M3</f>
-        <v>-0.86664023734398299</v>
+        <v>-6.0386232574100029E-3</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
+      <c r="B18" s="6">
+        <v>0.66524822695035402</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.89333333333333298</v>
+      </c>
+      <c r="D18" s="6">
+        <v>0.76260162601626003</v>
+      </c>
+      <c r="E18" s="6">
+        <v>0.74225319396051104</v>
+      </c>
+      <c r="F18" s="6">
+        <v>0.49712213913437497</v>
+      </c>
       <c r="G18" s="6">
         <f t="shared" ref="G18:G19" si="1">E18-M4</f>
-        <v>-0.75274706053833396</v>
+        <v>-1.0493866577822919E-2</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
+      <c r="B19" s="6">
+        <v>0.87956698240866005</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0.88075880758807501</v>
+      </c>
+      <c r="D19" s="6">
+        <v>0.88016249153689896</v>
+      </c>
+      <c r="E19" s="6">
+        <v>0.82986953966633203</v>
+      </c>
+      <c r="F19" s="6">
+        <v>0.65973936622283302</v>
+      </c>
       <c r="G19" s="6">
         <f t="shared" si="1"/>
-        <v>-0.82976738567267505</v>
+        <v>1.0215399365698374E-4</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -2631,37 +2701,37 @@
       <c r="F23" s="4"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
-      <c r="J24" s="13"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12" t="s">
+      <c r="C25" s="16"/>
+      <c r="D25" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12" t="s">
+      <c r="E25" s="16"/>
+      <c r="F25" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="G25" s="12"/>
-      <c r="I25" s="12" t="s">
+      <c r="G25" s="16"/>
+      <c r="I25" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="J25" s="12"/>
+      <c r="J25" s="16"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
@@ -2761,7 +2831,7 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
@@ -2770,8 +2840,10 @@
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
       <c r="H30" s="9"/>
-      <c r="I30" s="9"/>
-      <c r="J30" s="9"/>
+      <c r="I30" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J30" s="16"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
@@ -2784,33 +2856,136 @@
       <c r="D31" s="10" t="s">
         <v>18</v>
       </c>
+      <c r="I31" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J31" s="2">
+        <f>64*19</f>
+        <v>1216</v>
+      </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B32" s="2">
+        <v>2</v>
+      </c>
+      <c r="C32" s="2">
+        <v>9</v>
+      </c>
+      <c r="D32" s="2">
+        <v>26</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J32" s="2">
+        <f t="shared" ref="J32:J33" si="2">64*19</f>
+        <v>1216</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B33" s="2">
+        <v>1</v>
+      </c>
+      <c r="C33" s="2">
+        <v>4</v>
+      </c>
+      <c r="D33" s="2">
+        <v>20</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J33" s="2">
+        <f t="shared" si="2"/>
+        <v>1216</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
+      <c r="B34" s="2">
+        <v>1</v>
+      </c>
+      <c r="C34" s="2">
+        <v>7</v>
+      </c>
+      <c r="D34" s="2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B35" s="21"/>
+      <c r="C35" s="21"/>
+      <c r="D35" s="21"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="2"/>
+      <c r="B36" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B37" s="2">
+        <v>1</v>
+      </c>
+      <c r="C37" s="2">
+        <v>1</v>
+      </c>
+      <c r="D37" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B38" s="2">
+        <v>0</v>
+      </c>
+      <c r="C38" s="2">
+        <v>2</v>
+      </c>
+      <c r="D38" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B39" s="2">
+        <v>1</v>
+      </c>
+      <c r="C39" s="2">
+        <v>2</v>
+      </c>
+      <c r="D39" s="2">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="12">
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="I30:J30"/>
     <mergeCell ref="A30:D30"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="I1:N1"/>
@@ -2858,11 +3033,19 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1:G23">
-    <cfRule type="cellIs" dxfId="6" priority="5" operator="lessThan">
+  <conditionalFormatting sqref="B26:G28">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G1:G23">
+    <cfRule type="cellIs" dxfId="1" priority="5" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2878,14 +3061,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B26:G28">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>